<commit_message>
updated excel files with pf results from grids without trafo phase angles
</commit_message>
<xml_diff>
--- a/pandapower/test/shortcircuit/sce_tests/sc_result_comparison/wp_2.3/3_five_bus_radial_grid_1ph_dyn_MP_pf_sc_results_0_branch.xlsx
+++ b/pandapower/test/shortcircuit/sce_tests/sc_result_comparison/wp_2.3/3_five_bus_radial_grid_1ph_dyn_MP_pf_sc_results_0_branch.xlsx
@@ -876,40 +876,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.084258736675355E-14</v>
+        <v>-3.647452789181873E-14</v>
       </c>
       <c r="O2">
-        <v>3.126383720001767E-14</v>
+        <v>-1.042133752667725E-14</v>
       </c>
       <c r="P2">
-        <v>-4.453930233496634E-20</v>
+        <v>-4.453821947611989E-20</v>
       </c>
       <c r="Q2">
-        <v>1.042129368337693E-14</v>
+        <v>2.084258736675355E-14</v>
       </c>
       <c r="R2">
-        <v>-1.302614501157684E-14</v>
+        <v>2.344838287584099E-14</v>
       </c>
       <c r="S2">
-        <v>-5.210174055002065E-15</v>
+        <v>5.21111963228104E-15</v>
       </c>
       <c r="T2">
-        <v>5.210646841688128E-15</v>
+        <v>1.04212936833763E-14</v>
       </c>
       <c r="U2">
-        <v>5.763381835279506E-09</v>
+        <v>5.763394861896609E-09</v>
       </c>
       <c r="V2">
-        <v>-5.763397471383004E-09</v>
+        <v>-5.763407892676691E-09</v>
       </c>
       <c r="W2">
-        <v>-1.5631940525065E-14</v>
+        <v>-5.210646841688113E-15</v>
       </c>
       <c r="X2">
-        <v>-5.763394861410704E-09</v>
+        <v>-5.76339746673413E-09</v>
       </c>
       <c r="Y2">
-        <v>5.763402682515743E-09</v>
+        <v>5.763407893162593E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -933,37 +933,37 @@
         <v>1.100000023808766</v>
       </c>
       <c r="AG2">
-        <v>0.5500000117057466</v>
+        <v>0.5500000117057469</v>
       </c>
       <c r="AH2">
-        <v>0.550000012103019</v>
+        <v>0.5500000121030189</v>
       </c>
       <c r="AI2">
-        <v>1.100000023808766</v>
+        <v>1.100000023808765</v>
       </c>
       <c r="AJ2">
-        <v>0.550000011659377</v>
+        <v>0.5500000116593778</v>
       </c>
       <c r="AK2">
-        <v>0.5500000121493879</v>
+        <v>0.5500000121493883</v>
       </c>
       <c r="AL2">
-        <v>6.70306950820891E-13</v>
+        <v>7.005136949525866E-13</v>
       </c>
       <c r="AM2">
-        <v>-179.9999999995569</v>
+        <v>-179.9999999995568</v>
       </c>
       <c r="AN2">
         <v>179.9999999995499</v>
       </c>
       <c r="AO2">
-        <v>6.752509938312713E-13</v>
+        <v>7.077673301094281E-13</v>
       </c>
       <c r="AP2">
-        <v>-179.9999999952996</v>
+        <v>-179.9999999952994</v>
       </c>
       <c r="AQ2">
-        <v>179.9999999952925</v>
+        <v>179.9999999952926</v>
       </c>
     </row>
   </sheetData>
@@ -1148,40 +1148,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-5.210646841703823E-15</v>
+        <v>-1.04212936834076E-14</v>
       </c>
       <c r="O2">
-        <v>-7.307758498013522E-10</v>
+        <v>-7.30749227097718E-10</v>
       </c>
       <c r="P2">
-        <v>-2.039299493936969E-09</v>
+        <v>-2.039310370295516E-09</v>
       </c>
       <c r="Q2">
-        <v>-5.210646841703724E-15</v>
+        <v>5.008024835739682E-29</v>
       </c>
       <c r="R2">
-        <v>7.307806496600543E-10</v>
+        <v>7.307523449773011E-10</v>
       </c>
       <c r="S2">
-        <v>2.03929781224687E-09</v>
+        <v>2.039300316380309E-09</v>
       </c>
       <c r="T2">
-        <v>5.210646841703724E-15</v>
+        <v>5.210646841703675E-15</v>
       </c>
       <c r="U2">
-        <v>5.822509031582371E-09</v>
+        <v>5.822509524317716E-09</v>
       </c>
       <c r="V2">
-        <v>-3.556075895985844E-09</v>
+        <v>-3.556066663935935E-09</v>
       </c>
       <c r="W2">
-        <v>-5.210646841703825E-15</v>
+        <v>-5.210646841703774E-15</v>
       </c>
       <c r="X2">
-        <v>-5.822514425446013E-09</v>
+        <v>-5.822508683000228E-09</v>
       </c>
       <c r="Y2">
-        <v>3.556071710201213E-09</v>
+        <v>3.556065842109541E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -1205,37 +1205,37 @@
         <v>1.100000023812017</v>
       </c>
       <c r="AG2">
-        <v>0.6816683458635714</v>
+        <v>0.6816683458635716</v>
       </c>
       <c r="AH2">
-        <v>0.4761907155780343</v>
+        <v>0.4761907155780346</v>
       </c>
       <c r="AI2">
         <v>1.100000023812017</v>
       </c>
       <c r="AJ2">
-        <v>0.6816683458299556</v>
+        <v>0.6816683458299557</v>
       </c>
       <c r="AK2">
-        <v>0.476190715627781</v>
+        <v>0.4761907156277811</v>
       </c>
       <c r="AL2">
-        <v>5.468235264353422E-13</v>
+        <v>5.406519320173023E-13</v>
       </c>
       <c r="AM2">
-        <v>-164.9034422584275</v>
+        <v>-164.9034422584274</v>
       </c>
       <c r="AN2">
         <v>158.1097491654785</v>
       </c>
       <c r="AO2">
-        <v>5.556150992628499E-13</v>
+        <v>5.506776711252733E-13</v>
       </c>
       <c r="AP2">
         <v>-164.9034422552288</v>
       </c>
       <c r="AQ2">
-        <v>158.1097491642544</v>
+        <v>158.1097491642543</v>
       </c>
     </row>
   </sheetData>
@@ -1420,40 +1420,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-1.563194052511127E-14</v>
+        <v>-1.563194052511137E-14</v>
       </c>
       <c r="O2">
-        <v>-7.307883201636127E-10</v>
+        <v>-7.30765656040108E-10</v>
       </c>
       <c r="P2">
-        <v>-2.039317098211985E-09</v>
+        <v>-2.039314556408069E-09</v>
       </c>
       <c r="Q2">
-        <v>5.210646841703774E-15</v>
+        <v>5.210646841703825E-15</v>
       </c>
       <c r="R2">
-        <v>7.307985142138849E-10</v>
+        <v>7.307866384735204E-10</v>
       </c>
       <c r="S2">
-        <v>2.039314594367572E-09</v>
+        <v>2.039314556697087E-09</v>
       </c>
       <c r="T2">
-        <v>-5.210646841703924E-15</v>
+        <v>5.210646841703618E-15</v>
       </c>
       <c r="U2">
-        <v>5.822505667624132E-09</v>
+        <v>5.822508436960483E-09</v>
       </c>
       <c r="V2">
-        <v>-3.556083408386153E-09</v>
+        <v>-3.556064981956818E-09</v>
       </c>
       <c r="W2">
-        <v>5.111239790044058E-29</v>
+        <v>-5.21064684170372E-15</v>
       </c>
       <c r="X2">
-        <v>-5.82250626191809E-09</v>
+        <v>-5.822499432115079E-09</v>
       </c>
       <c r="Y2">
-        <v>3.556089276805751E-09</v>
+        <v>3.556064982284744E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -1477,34 +1477,34 @@
         <v>1.100000023812017</v>
       </c>
       <c r="AG2">
-        <v>0.6816683458635712</v>
+        <v>0.6816683458635716</v>
       </c>
       <c r="AH2">
-        <v>0.4761907155780346</v>
+        <v>0.4761907155780347</v>
       </c>
       <c r="AI2">
         <v>1.100000023812017</v>
       </c>
       <c r="AJ2">
-        <v>0.6816683458299556</v>
+        <v>0.6816683458299562</v>
       </c>
       <c r="AK2">
-        <v>0.4761907156277814</v>
+        <v>0.4761907156277815</v>
       </c>
       <c r="AL2">
-        <v>5.519312975242735E-13</v>
+        <v>5.703476357578039E-13</v>
       </c>
       <c r="AM2">
-        <v>-164.9034422584275</v>
+        <v>-164.9034422584274</v>
       </c>
       <c r="AN2">
-        <v>158.1097491654786</v>
+        <v>158.1097491654785</v>
       </c>
       <c r="AO2">
-        <v>5.620270898134577E-13</v>
+        <v>5.769013612765529E-13</v>
       </c>
       <c r="AP2">
-        <v>-164.9034422552288</v>
+        <v>-164.9034422552287</v>
       </c>
       <c r="AQ2">
         <v>158.1097491642544</v>
@@ -1692,40 +1692,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-7.105427357603425E-15</v>
+        <v>-2.36847578586779E-15</v>
       </c>
       <c r="O2">
-        <v>-5.92129177239103E-15</v>
+        <v>2.368373474356434E-15</v>
       </c>
       <c r="P2">
-        <v>2.368372904615314E-15</v>
+        <v>4.736848688587432E-15</v>
       </c>
       <c r="Q2">
-        <v>9.473903143471389E-15</v>
+        <v>4.736951571735584E-15</v>
       </c>
       <c r="R2">
-        <v>5.921971311542139E-15</v>
+        <v>2.369257632397851E-15</v>
       </c>
       <c r="S2">
-        <v>4.737733992697316E-15</v>
+        <v>2.369258204205662E-15</v>
       </c>
       <c r="T2">
-        <v>-9.473903143471473E-15</v>
+        <v>-4.736951571735722E-15</v>
       </c>
       <c r="U2">
-        <v>4.763144543706228E-09</v>
+        <v>4.76313033285152E-09</v>
       </c>
       <c r="V2">
-        <v>-4.763146915672772E-09</v>
+        <v>-4.763127967866474E-09</v>
       </c>
       <c r="W2">
-        <v>1.145331320840004E-28</v>
+        <v>9.473903143471448E-15</v>
       </c>
       <c r="X2">
-        <v>-4.763146911780441E-09</v>
+        <v>-4.763135069401517E-09</v>
       </c>
       <c r="Y2">
-        <v>4.763142179122765E-09</v>
+        <v>4.763132705219609E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -1749,22 +1749,22 @@
         <v>1.000000000000357</v>
       </c>
       <c r="AG2">
-        <v>0.4999999998169616</v>
+        <v>0.4999999998169618</v>
       </c>
       <c r="AH2">
-        <v>0.5000000001833957</v>
+        <v>0.5000000001833953</v>
       </c>
       <c r="AI2">
-        <v>1.000000000000357</v>
+        <v>1.000000000000358</v>
       </c>
       <c r="AJ2">
-        <v>0.4999999997748078</v>
+        <v>0.4999999997748076</v>
       </c>
       <c r="AK2">
-        <v>0.5000000002255494</v>
+        <v>0.5000000002255485</v>
       </c>
       <c r="AL2">
-        <v>6.98880354923979E-13</v>
+        <v>6.876682335354553E-13</v>
       </c>
       <c r="AM2">
         <v>-179.999999998762</v>
@@ -1773,7 +1773,7 @@
         <v>179.9999999987551</v>
       </c>
       <c r="AO2">
-        <v>6.92667529258995E-13</v>
+        <v>6.748009875736533E-13</v>
       </c>
       <c r="AP2">
         <v>-179.9999999905878</v>
@@ -1964,40 +1964,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-7.105427357603425E-15</v>
+        <v>-2.36847578586779E-15</v>
       </c>
       <c r="O2">
-        <v>-5.92129177239103E-15</v>
+        <v>2.368373474356434E-15</v>
       </c>
       <c r="P2">
-        <v>2.368372904615314E-15</v>
+        <v>4.736848688587432E-15</v>
       </c>
       <c r="Q2">
-        <v>9.473903143471389E-15</v>
+        <v>4.736951571735584E-15</v>
       </c>
       <c r="R2">
-        <v>5.921971311542139E-15</v>
+        <v>2.369257632397851E-15</v>
       </c>
       <c r="S2">
-        <v>4.737733992697316E-15</v>
+        <v>2.369258204205662E-15</v>
       </c>
       <c r="T2">
-        <v>-9.473903143471473E-15</v>
+        <v>-4.736951571735722E-15</v>
       </c>
       <c r="U2">
-        <v>4.763144543706228E-09</v>
+        <v>4.76313033285152E-09</v>
       </c>
       <c r="V2">
-        <v>-4.763146915672772E-09</v>
+        <v>-4.763127967866474E-09</v>
       </c>
       <c r="W2">
-        <v>1.145331320840004E-28</v>
+        <v>9.473903143471448E-15</v>
       </c>
       <c r="X2">
-        <v>-4.763146911780441E-09</v>
+        <v>-4.763135069401517E-09</v>
       </c>
       <c r="Y2">
-        <v>4.763142179122765E-09</v>
+        <v>4.763132705219609E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -2021,22 +2021,22 @@
         <v>1.000000000000357</v>
       </c>
       <c r="AG2">
-        <v>0.4999999998169616</v>
+        <v>0.4999999998169618</v>
       </c>
       <c r="AH2">
-        <v>0.5000000001833957</v>
+        <v>0.5000000001833953</v>
       </c>
       <c r="AI2">
-        <v>1.000000000000357</v>
+        <v>1.000000000000358</v>
       </c>
       <c r="AJ2">
-        <v>0.4999999997748078</v>
+        <v>0.4999999997748076</v>
       </c>
       <c r="AK2">
-        <v>0.5000000002255494</v>
+        <v>0.5000000002255485</v>
       </c>
       <c r="AL2">
-        <v>6.98880354923979E-13</v>
+        <v>6.876682335354553E-13</v>
       </c>
       <c r="AM2">
         <v>-179.999999998762</v>
@@ -2045,7 +2045,7 @@
         <v>179.9999999987551</v>
       </c>
       <c r="AO2">
-        <v>6.92667529258995E-13</v>
+        <v>6.748009875736533E-13</v>
       </c>
       <c r="AP2">
         <v>-179.9999999905878</v>
@@ -2236,40 +2236,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-9.473903143522943E-15</v>
+        <v>-4.736951571761458E-15</v>
       </c>
       <c r="O2">
-        <v>-5.559639858305625E-10</v>
+        <v>-5.559594148032301E-10</v>
       </c>
       <c r="P2">
-        <v>-1.551464144763422E-09</v>
+        <v>-1.551456171948549E-09</v>
       </c>
       <c r="Q2">
-        <v>7.105427357642179E-15</v>
+        <v>4.736951571761484E-15</v>
       </c>
       <c r="R2">
-        <v>5.559698875872633E-10</v>
+        <v>5.559653165599338E-10</v>
       </c>
       <c r="S2">
-        <v>1.551466660388596E-09</v>
+        <v>1.551461416408438E-09</v>
       </c>
       <c r="T2">
-        <v>-2.368475785880837E-15</v>
+        <v>-2.368475785880789E-15</v>
       </c>
       <c r="U2">
-        <v>4.833167299792688E-09</v>
+        <v>4.833172859965311E-09</v>
       </c>
       <c r="V2">
-        <v>-3.108913797919907E-09</v>
+        <v>-3.108903523648881E-09</v>
       </c>
       <c r="W2">
-        <v>4.736951571761556E-15</v>
+        <v>4.642443535461416E-29</v>
       </c>
       <c r="X2">
-        <v>-4.833173269121602E-09</v>
+        <v>-4.833178829294224E-09</v>
       </c>
       <c r="Y2">
-        <v>3.10890855422325E-09</v>
+        <v>3.10890603907781E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -2290,25 +2290,25 @@
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>1.000000000005802</v>
+        <v>1.000000000005801</v>
       </c>
       <c r="AG2">
-        <v>0.6078088903891383</v>
+        <v>0.6078088903891384</v>
       </c>
       <c r="AH2">
-        <v>0.4340870104140602</v>
+        <v>0.4340870104140598</v>
       </c>
       <c r="AI2">
         <v>1.000000000005802</v>
       </c>
       <c r="AJ2">
-        <v>0.6078088903608007</v>
+        <v>0.6078088903608005</v>
       </c>
       <c r="AK2">
-        <v>0.4340870104725144</v>
+        <v>0.4340870104725136</v>
       </c>
       <c r="AL2">
-        <v>5.803130044823412E-13</v>
+        <v>5.753611481049673E-13</v>
       </c>
       <c r="AM2">
         <v>-166.2935793302449</v>
@@ -2317,7 +2317,7 @@
         <v>160.6235536346806</v>
       </c>
       <c r="AO2">
-        <v>5.789459946013811E-13</v>
+        <v>5.61526579235871E-13</v>
       </c>
       <c r="AP2">
         <v>-166.2935793242505</v>
@@ -2508,40 +2508,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-9.473903143522943E-15</v>
+        <v>-4.736951571761458E-15</v>
       </c>
       <c r="O2">
-        <v>-5.559639858305625E-10</v>
+        <v>-5.559594148032301E-10</v>
       </c>
       <c r="P2">
-        <v>-1.551464144763422E-09</v>
+        <v>-1.551456171948549E-09</v>
       </c>
       <c r="Q2">
-        <v>7.105427357642179E-15</v>
+        <v>4.736951571761484E-15</v>
       </c>
       <c r="R2">
-        <v>5.559698875872633E-10</v>
+        <v>5.559653165599338E-10</v>
       </c>
       <c r="S2">
-        <v>1.551466660388596E-09</v>
+        <v>1.551461416408438E-09</v>
       </c>
       <c r="T2">
-        <v>-2.368475785880837E-15</v>
+        <v>-2.368475785880789E-15</v>
       </c>
       <c r="U2">
-        <v>4.833167299792688E-09</v>
+        <v>4.833172859965311E-09</v>
       </c>
       <c r="V2">
-        <v>-3.108913797919907E-09</v>
+        <v>-3.108903523648881E-09</v>
       </c>
       <c r="W2">
-        <v>4.736951571761556E-15</v>
+        <v>4.642443535461416E-29</v>
       </c>
       <c r="X2">
-        <v>-4.833173269121602E-09</v>
+        <v>-4.833178829294224E-09</v>
       </c>
       <c r="Y2">
-        <v>3.10890855422325E-09</v>
+        <v>3.10890603907781E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -2562,25 +2562,25 @@
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>1.000000000005802</v>
+        <v>1.000000000005801</v>
       </c>
       <c r="AG2">
-        <v>0.6078088903891383</v>
+        <v>0.6078088903891384</v>
       </c>
       <c r="AH2">
-        <v>0.4340870104140602</v>
+        <v>0.4340870104140598</v>
       </c>
       <c r="AI2">
         <v>1.000000000005802</v>
       </c>
       <c r="AJ2">
-        <v>0.6078088903608007</v>
+        <v>0.6078088903608005</v>
       </c>
       <c r="AK2">
-        <v>0.4340870104725144</v>
+        <v>0.4340870104725136</v>
       </c>
       <c r="AL2">
-        <v>5.803130044823412E-13</v>
+        <v>5.753611481049673E-13</v>
       </c>
       <c r="AM2">
         <v>-166.2935793302449</v>
@@ -2589,7 +2589,7 @@
         <v>160.6235536346806</v>
       </c>
       <c r="AO2">
-        <v>5.789459946013811E-13</v>
+        <v>5.61526579235871E-13</v>
       </c>
       <c r="AP2">
         <v>-166.2935793242505</v>
@@ -2783,40 +2783,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.957776350055461E-09</v>
+        <v>-2.957783297584583E-09</v>
       </c>
       <c r="O2">
-        <v>-7.394557797340441E-10</v>
+        <v>-7.394502283935339E-10</v>
       </c>
       <c r="P2">
-        <v>-7.394257116383617E-10</v>
+        <v>-7.394616417118109E-10</v>
       </c>
       <c r="Q2">
-        <v>2.957775047647529E-09</v>
+        <v>2.95778286361779E-09</v>
       </c>
       <c r="R2">
-        <v>7.394555626872028E-10</v>
+        <v>7.39448925795268E-10</v>
       </c>
       <c r="S2">
-        <v>7.394392493594112E-10</v>
+        <v>7.394652858866506E-10</v>
       </c>
       <c r="T2">
-        <v>1.215731871110989E-14</v>
+        <v>-1.737739537755098E-15</v>
       </c>
       <c r="U2">
-        <v>-3.842251992236992E-09</v>
+        <v>-3.842271779329416E-09</v>
       </c>
       <c r="V2">
-        <v>3.842265967863286E-09</v>
+        <v>3.842282451537977E-09</v>
       </c>
       <c r="W2">
-        <v>-1.21570307703489E-14</v>
+        <v>5.211792039058353E-15</v>
       </c>
       <c r="X2">
-        <v>3.842250864170842E-09</v>
+        <v>3.842265010572598E-09</v>
       </c>
       <c r="Y2">
-        <v>-3.84226336246788E-09</v>
+        <v>-3.842277070472316E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -2837,40 +2837,40 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.3666666746541449</v>
+        <v>0.3666666746541453</v>
       </c>
       <c r="AH2">
-        <v>0.9701088351760906</v>
+        <v>0.9701088351760907</v>
       </c>
       <c r="AI2">
-        <v>0.9701088350717374</v>
+        <v>0.9701088350717375</v>
       </c>
       <c r="AJ2">
-        <v>0.3666666746856049</v>
+        <v>0.3666666746856054</v>
       </c>
       <c r="AK2">
-        <v>0.9701088351965889</v>
+        <v>0.9701088351965894</v>
       </c>
       <c r="AL2">
-        <v>0.9701088350571845</v>
+        <v>0.9701088350571841</v>
       </c>
       <c r="AM2">
-        <v>1.660607855946246E-08</v>
+        <v>1.660608646149717E-08</v>
       </c>
       <c r="AN2">
         <v>-100.8933946492837</v>
       </c>
       <c r="AO2">
-        <v>100.8933946504708</v>
+        <v>100.8933946504709</v>
       </c>
       <c r="AP2">
-        <v>2.218387656172014E-08</v>
+        <v>2.218381528064411E-08</v>
       </c>
       <c r="AQ2">
         <v>-100.8933946499968</v>
       </c>
       <c r="AR2">
-        <v>100.8933946515823</v>
+        <v>100.8933946515824</v>
       </c>
     </row>
   </sheetData>
@@ -3058,40 +3058,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.957770705188049E-09</v>
+        <v>-2.957775047393748E-09</v>
       </c>
       <c r="O2">
-        <v>-7.394367759093438E-10</v>
+        <v>-7.394410713515951E-10</v>
       </c>
       <c r="P2">
-        <v>-7.394454987307843E-10</v>
+        <v>-7.394257116383612E-10</v>
       </c>
       <c r="Q2">
-        <v>2.957773310765246E-09</v>
+        <v>2.957771139662391E-09</v>
       </c>
       <c r="R2">
-        <v>7.394389470756403E-10</v>
+        <v>7.394383809182014E-10</v>
       </c>
       <c r="S2">
-        <v>7.394590364518355E-10</v>
+        <v>7.394338683657355E-10</v>
       </c>
       <c r="T2">
-        <v>6.946671870465632E-15</v>
+        <v>5.209789589081567E-15</v>
       </c>
       <c r="U2">
-        <v>-3.842262669050926E-09</v>
+        <v>-3.842260672471653E-09</v>
       </c>
       <c r="V2">
-        <v>3.842271519203792E-09</v>
+        <v>3.842265967863286E-09</v>
       </c>
       <c r="W2">
-        <v>-8.683266211379656E-15</v>
+        <v>1.738027472027629E-15</v>
       </c>
       <c r="X2">
-        <v>3.84227395050425E-09</v>
+        <v>3.842258850487939E-09</v>
       </c>
       <c r="Y2">
-        <v>-3.842268913808386E-09</v>
+        <v>-3.842259718356485E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -3112,13 +3112,13 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.3666666746541452</v>
+        <v>0.3666666746541449</v>
       </c>
       <c r="AH2">
         <v>0.9701088351760905</v>
       </c>
       <c r="AI2">
-        <v>0.9701088350717373</v>
+        <v>0.9701088350717374</v>
       </c>
       <c r="AJ2">
         <v>0.3666666746856049</v>
@@ -3127,25 +3127,25 @@
         <v>0.970108835196589</v>
       </c>
       <c r="AL2">
-        <v>0.9701088350571843</v>
+        <v>0.9701088350571841</v>
       </c>
       <c r="AM2">
-        <v>1.660607592545088E-08</v>
+        <v>1.660606275539302E-08</v>
       </c>
       <c r="AN2">
         <v>-100.8933946492837</v>
       </c>
       <c r="AO2">
-        <v>100.8933946504709</v>
+        <v>100.8933946504708</v>
       </c>
       <c r="AP2">
-        <v>2.218383264354411E-08</v>
+        <v>2.218380399653162E-08</v>
       </c>
       <c r="AQ2">
         <v>-100.8933946499968</v>
       </c>
       <c r="AR2">
-        <v>100.8933946515824</v>
+        <v>100.8933946515823</v>
       </c>
     </row>
   </sheetData>
@@ -3333,40 +3333,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-3.138984078360133E-09</v>
+        <v>-3.138990760387152E-09</v>
       </c>
       <c r="O2">
-        <v>-1.398932104635029E-09</v>
+        <v>-1.398932508406665E-09</v>
       </c>
       <c r="P2">
-        <v>-1.70568933393092E-10</v>
+        <v>-1.70574209892848E-10</v>
       </c>
       <c r="Q2">
-        <v>3.138984191042502E-09</v>
+        <v>3.138990760507736E-09</v>
       </c>
       <c r="R2">
-        <v>1.398929921813651E-09</v>
+        <v>1.398922958080293E-09</v>
       </c>
       <c r="S2">
-        <v>1.70577073101277E-10</v>
+        <v>1.70579000113179E-10</v>
       </c>
       <c r="T2">
-        <v>1.418396439578959E-09</v>
+        <v>1.418385026522095E-09</v>
       </c>
       <c r="U2">
-        <v>-2.221735843084712E-09</v>
+        <v>-2.221743974536927E-09</v>
       </c>
       <c r="V2">
-        <v>2.930924681608889E-09</v>
+        <v>2.930933541638094E-09</v>
       </c>
       <c r="W2">
-        <v>-1.418391978516324E-09</v>
+        <v>-1.418385026385279E-09</v>
       </c>
       <c r="X2">
-        <v>2.22172595438484E-09</v>
+        <v>2.221743679789629E-09</v>
       </c>
       <c r="Y2">
-        <v>-2.930917009979838E-09</v>
+        <v>-2.930932100901559E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -3387,19 +3387,19 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.619474449769583</v>
+        <v>0.6194744497695832</v>
       </c>
       <c r="AH2">
-        <v>0.94433477094435</v>
+        <v>0.9443347709443498</v>
       </c>
       <c r="AI2">
         <v>1.05598589769414</v>
       </c>
       <c r="AJ2">
-        <v>0.6194744497792133</v>
+        <v>0.6194744497792136</v>
       </c>
       <c r="AK2">
-        <v>0.9443347709605379</v>
+        <v>0.9443347709605382</v>
       </c>
       <c r="AL2">
         <v>1.055985897682488</v>
@@ -3414,7 +3414,7 @@
         <v>106.7392371168768</v>
       </c>
       <c r="AP2">
-        <v>-10.90775017560494</v>
+        <v>-10.90775017560496</v>
       </c>
       <c r="AQ2">
         <v>-108.7881138043734</v>
@@ -3724,40 +3724,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-3.138979756253142E-09</v>
+        <v>-3.138985076348948E-09</v>
       </c>
       <c r="O2">
-        <v>-1.398926789193395E-09</v>
+        <v>-1.398921495549789E-09</v>
       </c>
       <c r="P2">
-        <v>-1.705756505951787E-10</v>
+        <v>-1.705531221202049E-10</v>
       </c>
       <c r="Q2">
-        <v>3.138980146573159E-09</v>
+        <v>3.138984607498975E-09</v>
       </c>
       <c r="R2">
-        <v>1.398928906680984E-09</v>
+        <v>1.398927509574707E-09</v>
       </c>
       <c r="S2">
-        <v>1.705708604351399E-10</v>
+        <v>1.705593530428672E-10</v>
       </c>
       <c r="T2">
-        <v>1.41839560666601E-09</v>
+        <v>1.418395137695454E-09</v>
       </c>
       <c r="U2">
-        <v>-2.221734107600879E-09</v>
+        <v>-2.221735908478793E-09</v>
       </c>
       <c r="V2">
-        <v>2.930938331828279E-09</v>
+        <v>2.930924213525697E-09</v>
       </c>
       <c r="W2">
-        <v>-1.418389704901044E-09</v>
+        <v>-1.418389817462829E-09</v>
       </c>
       <c r="X2">
-        <v>2.221733387283917E-09</v>
+        <v>2.221736225092525E-09</v>
       </c>
       <c r="Y2">
-        <v>-2.930939772496407E-09</v>
+        <v>-2.930927562979348E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -3778,25 +3778,25 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.6194744497695832</v>
+        <v>0.619474449769583</v>
       </c>
       <c r="AH2">
-        <v>0.9443347709443497</v>
+        <v>0.9443347709443498</v>
       </c>
       <c r="AI2">
         <v>1.05598589769414</v>
       </c>
       <c r="AJ2">
-        <v>0.6194744497792134</v>
+        <v>0.6194744497792132</v>
       </c>
       <c r="AK2">
-        <v>0.9443347709605379</v>
+        <v>0.9443347709605381</v>
       </c>
       <c r="AL2">
         <v>1.055985897682488</v>
       </c>
       <c r="AM2">
-        <v>-10.90775017850473</v>
+        <v>-10.90775017850475</v>
       </c>
       <c r="AN2">
         <v>-108.7881138042144</v>
@@ -3805,7 +3805,7 @@
         <v>106.7392371168768</v>
       </c>
       <c r="AP2">
-        <v>-10.90775017560496</v>
+        <v>-10.90775017560498</v>
       </c>
       <c r="AQ2">
         <v>-108.7881138043734</v>
@@ -3999,40 +3999,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.444445830918463E-09</v>
+        <v>-2.4444454361725E-09</v>
       </c>
       <c r="O2">
-        <v>-6.111050469047306E-10</v>
+        <v>-6.111039826094429E-10</v>
       </c>
       <c r="P2">
-        <v>-6.111117537891439E-10</v>
+        <v>-6.111199584299389E-10</v>
       </c>
       <c r="Q2">
-        <v>2.444443462845366E-09</v>
+        <v>2.444448989288868E-09</v>
       </c>
       <c r="R2">
-        <v>6.111065060466547E-10</v>
+        <v>6.111009059698166E-10</v>
       </c>
       <c r="S2">
-        <v>6.111097027296174E-10</v>
+        <v>6.111171178784836E-10</v>
       </c>
       <c r="T2">
-        <v>-7.898461213897504E-16</v>
+        <v>1.578629665359891E-15</v>
       </c>
       <c r="U2">
-        <v>-3.175422602320105E-09</v>
+        <v>-3.175428124966566E-09</v>
       </c>
       <c r="V2">
-        <v>3.175429819918893E-09</v>
+        <v>3.175428240935037E-09</v>
       </c>
       <c r="W2">
-        <v>-7.888997702829614E-16</v>
+        <v>-1.183645732986666E-15</v>
       </c>
       <c r="X2">
-        <v>3.175419130893334E-09</v>
+        <v>3.175428717145004E-09</v>
       </c>
       <c r="Y2">
-        <v>-3.175430214605366E-09</v>
+        <v>-3.175424533301113E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -4053,37 +4053,37 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.3333333333308632</v>
+        <v>0.3333333333308633</v>
       </c>
       <c r="AH2">
-        <v>0.8819171037085271</v>
+        <v>0.8819171037085273</v>
       </c>
       <c r="AI2">
-        <v>0.8819171036611017</v>
+        <v>0.8819171036611018</v>
       </c>
       <c r="AJ2">
-        <v>0.3333333333857753</v>
+        <v>0.3333333333857754</v>
       </c>
       <c r="AK2">
-        <v>0.8819171037296484</v>
+        <v>0.8819171037296483</v>
       </c>
       <c r="AL2">
-        <v>0.8819171036503577</v>
+        <v>0.881917103650358</v>
       </c>
       <c r="AM2">
-        <v>8.301984353899825E-09</v>
+        <v>8.301964594821198E-09</v>
       </c>
       <c r="AN2">
-        <v>-100.8933946487908</v>
+        <v>-100.8933946487909</v>
       </c>
       <c r="AO2">
         <v>100.8933946493849</v>
       </c>
       <c r="AP2">
-        <v>1.387971588697872E-08</v>
+        <v>1.387972364072079E-08</v>
       </c>
       <c r="AQ2">
-        <v>-100.8933946503432</v>
+        <v>-100.8933946503433</v>
       </c>
       <c r="AR2">
         <v>100.8933946513357</v>
@@ -4274,40 +4274,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.444445830918463E-09</v>
+        <v>-2.4444454361725E-09</v>
       </c>
       <c r="O2">
-        <v>-6.111050469047306E-10</v>
+        <v>-6.111039826094429E-10</v>
       </c>
       <c r="P2">
-        <v>-6.111117537891439E-10</v>
+        <v>-6.111199584299389E-10</v>
       </c>
       <c r="Q2">
-        <v>2.444443462845366E-09</v>
+        <v>2.444448989288868E-09</v>
       </c>
       <c r="R2">
-        <v>6.111065060466547E-10</v>
+        <v>6.111009059698166E-10</v>
       </c>
       <c r="S2">
-        <v>6.111097027296174E-10</v>
+        <v>6.111171178784836E-10</v>
       </c>
       <c r="T2">
-        <v>-7.898461213897504E-16</v>
+        <v>1.578629665359891E-15</v>
       </c>
       <c r="U2">
-        <v>-3.175422602320105E-09</v>
+        <v>-3.175428124966566E-09</v>
       </c>
       <c r="V2">
-        <v>3.175429819918893E-09</v>
+        <v>3.175428240935037E-09</v>
       </c>
       <c r="W2">
-        <v>-7.888997702829614E-16</v>
+        <v>-1.183645732986666E-15</v>
       </c>
       <c r="X2">
-        <v>3.175419130893334E-09</v>
+        <v>3.175428717145004E-09</v>
       </c>
       <c r="Y2">
-        <v>-3.175430214605366E-09</v>
+        <v>-3.175424533301113E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -4328,37 +4328,37 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.3333333333308632</v>
+        <v>0.3333333333308633</v>
       </c>
       <c r="AH2">
-        <v>0.8819171037085271</v>
+        <v>0.8819171037085273</v>
       </c>
       <c r="AI2">
-        <v>0.8819171036611017</v>
+        <v>0.8819171036611018</v>
       </c>
       <c r="AJ2">
-        <v>0.3333333333857753</v>
+        <v>0.3333333333857754</v>
       </c>
       <c r="AK2">
-        <v>0.8819171037296484</v>
+        <v>0.8819171037296483</v>
       </c>
       <c r="AL2">
-        <v>0.8819171036503577</v>
+        <v>0.881917103650358</v>
       </c>
       <c r="AM2">
-        <v>8.301984353899825E-09</v>
+        <v>8.301964594821198E-09</v>
       </c>
       <c r="AN2">
-        <v>-100.8933946487908</v>
+        <v>-100.8933946487909</v>
       </c>
       <c r="AO2">
         <v>100.8933946493849</v>
       </c>
       <c r="AP2">
-        <v>1.387971588697872E-08</v>
+        <v>1.387972364072079E-08</v>
       </c>
       <c r="AQ2">
-        <v>-100.8933946503432</v>
+        <v>-100.8933946503433</v>
       </c>
       <c r="AR2">
         <v>100.8933946513357</v>
@@ -4549,40 +4549,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.62475477461107E-09</v>
+        <v>-2.624757566945495E-09</v>
       </c>
       <c r="O2">
-        <v>-1.140201278215544E-09</v>
+        <v>-1.140198381982747E-09</v>
       </c>
       <c r="P2">
-        <v>-1.721708307665985E-10</v>
+        <v>-1.721816882592633E-10</v>
       </c>
       <c r="Q2">
-        <v>2.624753903471849E-09</v>
+        <v>2.624757807829497E-09</v>
       </c>
       <c r="R2">
-        <v>1.140199662780455E-09</v>
+        <v>1.140198510592896E-09</v>
       </c>
       <c r="S2">
-        <v>1.721695694786605E-10</v>
+        <v>1.7218060256183E-10</v>
       </c>
       <c r="T2">
-        <v>1.117783161330853E-09</v>
+        <v>1.117785655032181E-09</v>
       </c>
       <c r="U2">
-        <v>-1.947063510543381E-09</v>
+        <v>-1.94706445654821E-09</v>
       </c>
       <c r="V2">
-        <v>2.505961007446678E-09</v>
+        <v>2.50595785409725E-09</v>
       </c>
       <c r="W2">
-        <v>-1.117784302209768E-09</v>
+        <v>-1.117784393569887E-09</v>
       </c>
       <c r="X2">
-        <v>1.947065106654829E-09</v>
+        <v>1.947069756635915E-09</v>
       </c>
       <c r="Y2">
-        <v>-2.505956664418982E-09</v>
+        <v>-2.505958169401564E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -4615,13 +4615,13 @@
         <v>0.5421614591770477</v>
       </c>
       <c r="AK2">
-        <v>0.8576025463355479</v>
+        <v>0.8576025463355478</v>
       </c>
       <c r="AL2">
-        <v>0.9547184906556984</v>
+        <v>0.9547184906556988</v>
       </c>
       <c r="AM2">
-        <v>-10.80277169403304</v>
+        <v>-10.80277169403305</v>
       </c>
       <c r="AN2">
         <v>-108.0887396155923</v>
@@ -4630,13 +4630,13 @@
         <v>106.1949204558219</v>
       </c>
       <c r="AP2">
-        <v>-10.80277169013759</v>
+        <v>-10.80277169013758</v>
       </c>
       <c r="AQ2">
         <v>-108.0887396163351</v>
       </c>
       <c r="AR2">
-        <v>106.1949204570493</v>
+        <v>106.1949204570494</v>
       </c>
     </row>
   </sheetData>
@@ -4824,40 +4824,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.62475477461107E-09</v>
+        <v>-2.624757566945495E-09</v>
       </c>
       <c r="O2">
-        <v>-1.140201278215544E-09</v>
+        <v>-1.140198381982747E-09</v>
       </c>
       <c r="P2">
-        <v>-1.721708307665985E-10</v>
+        <v>-1.721816882592633E-10</v>
       </c>
       <c r="Q2">
-        <v>2.624753903471849E-09</v>
+        <v>2.624757807829497E-09</v>
       </c>
       <c r="R2">
-        <v>1.140199662780455E-09</v>
+        <v>1.140198510592896E-09</v>
       </c>
       <c r="S2">
-        <v>1.721695694786605E-10</v>
+        <v>1.7218060256183E-10</v>
       </c>
       <c r="T2">
-        <v>1.117783161330853E-09</v>
+        <v>1.117785655032181E-09</v>
       </c>
       <c r="U2">
-        <v>-1.947063510543381E-09</v>
+        <v>-1.94706445654821E-09</v>
       </c>
       <c r="V2">
-        <v>2.505961007446678E-09</v>
+        <v>2.50595785409725E-09</v>
       </c>
       <c r="W2">
-        <v>-1.117784302209768E-09</v>
+        <v>-1.117784393569887E-09</v>
       </c>
       <c r="X2">
-        <v>1.947065106654829E-09</v>
+        <v>1.947069756635915E-09</v>
       </c>
       <c r="Y2">
-        <v>-2.505956664418982E-09</v>
+        <v>-2.505958169401564E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -4890,13 +4890,13 @@
         <v>0.5421614591770477</v>
       </c>
       <c r="AK2">
-        <v>0.8576025463355479</v>
+        <v>0.8576025463355478</v>
       </c>
       <c r="AL2">
-        <v>0.9547184906556984</v>
+        <v>0.9547184906556988</v>
       </c>
       <c r="AM2">
-        <v>-10.80277169403304</v>
+        <v>-10.80277169403305</v>
       </c>
       <c r="AN2">
         <v>-108.0887396155923</v>
@@ -4905,13 +4905,13 @@
         <v>106.1949204558219</v>
       </c>
       <c r="AP2">
-        <v>-10.80277169013759</v>
+        <v>-10.80277169013758</v>
       </c>
       <c r="AQ2">
         <v>-108.0887396163351</v>
       </c>
       <c r="AR2">
-        <v>106.1949204570493</v>
+        <v>106.1949204570494</v>
       </c>
     </row>
   </sheetData>
@@ -5099,40 +5099,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.957775046935625E-09</v>
+        <v>-2.957788941993869E-09</v>
       </c>
       <c r="O2">
-        <v>-7.394324716518695E-10</v>
+        <v>-7.394307347695905E-10</v>
       </c>
       <c r="P2">
-        <v>-7.394533148874835E-10</v>
+        <v>-7.394463673583611E-10</v>
       </c>
       <c r="Q2">
-        <v>2.957768099469948E-09</v>
+        <v>2.957781994528193E-09</v>
       </c>
       <c r="R2">
-        <v>7.394411565073724E-10</v>
+        <v>7.394394196250955E-10</v>
       </c>
       <c r="S2">
-        <v>7.394359465087788E-10</v>
+        <v>7.394463678024713E-10</v>
       </c>
       <c r="T2">
-        <v>1.042121706896095E-14</v>
+        <v>-3.473841175078359E-15</v>
       </c>
       <c r="U2">
-        <v>3.842258029733097E-09</v>
+        <v>3.842258029733095E-09</v>
       </c>
       <c r="V2">
-        <v>-3.842261507934168E-09</v>
+        <v>-3.842268455463296E-09</v>
       </c>
       <c r="W2">
-        <v>1.485997317519135E-19</v>
+        <v>1.389520684364833E-14</v>
       </c>
       <c r="X2">
-        <v>-3.842256292346922E-09</v>
+        <v>-3.842259766111477E-09</v>
       </c>
       <c r="Y2">
-        <v>3.842261508438059E-09</v>
+        <v>3.842261508438062E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -5156,31 +5156,31 @@
         <v>0.7333333491947058</v>
       </c>
       <c r="AH2">
-        <v>0.3666666743874889</v>
+        <v>0.3666666743874887</v>
       </c>
       <c r="AI2">
-        <v>0.3666666748072245</v>
+        <v>0.3666666748072248</v>
       </c>
       <c r="AJ2">
-        <v>0.733333349210436</v>
+        <v>0.7333333492104364</v>
       </c>
       <c r="AK2">
-        <v>0.3666666743489845</v>
+        <v>0.3666666743489841</v>
       </c>
       <c r="AL2">
-        <v>0.3666666748614584</v>
+        <v>0.3666666748614587</v>
       </c>
       <c r="AM2">
-        <v>1.484113408313245E-09</v>
+        <v>1.484101555261158E-09</v>
       </c>
       <c r="AN2">
         <v>-179.9999999988593</v>
       </c>
       <c r="AO2">
-        <v>-179.9999999981703</v>
+        <v>-179.9999999981704</v>
       </c>
       <c r="AP2">
-        <v>2.878568291978759E-09</v>
+        <v>2.878541736845484E-09</v>
       </c>
       <c r="AQ2">
         <v>-179.9999999910789</v>
@@ -5374,40 +5374,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.957788941993869E-09</v>
+        <v>-2.957785468229309E-09</v>
       </c>
       <c r="O2">
-        <v>-7.394342085341486E-10</v>
+        <v>-7.394463667101141E-10</v>
       </c>
       <c r="P2">
-        <v>-7.394533148874854E-10</v>
+        <v>-7.394463673583575E-10</v>
       </c>
       <c r="Q2">
-        <v>2.957781994528193E-09</v>
+        <v>2.957778520763631E-09</v>
       </c>
       <c r="R2">
-        <v>7.394498409187727E-10</v>
+        <v>7.39455051565621E-10</v>
       </c>
       <c r="S2">
-        <v>7.394359465087802E-10</v>
+        <v>7.394498415670336E-10</v>
       </c>
       <c r="T2">
-        <v>-3.473841176064185E-15</v>
+        <v>6.947452505136632E-15</v>
       </c>
       <c r="U2">
-        <v>3.842263240379933E-09</v>
+        <v>3.842264977262214E-09</v>
       </c>
       <c r="V2">
-        <v>-3.842261507934172E-09</v>
+        <v>-3.84226150793417E-09</v>
       </c>
       <c r="W2">
-        <v>3.473913161687661E-15</v>
+        <v>1.486022671732196E-19</v>
       </c>
       <c r="X2">
-        <v>-3.842266713640593E-09</v>
+        <v>-3.842264976758318E-09</v>
       </c>
       <c r="Y2">
-        <v>3.842268455967191E-09</v>
+        <v>3.842275403496318E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -5431,34 +5431,34 @@
         <v>0.7333333491947058</v>
       </c>
       <c r="AH2">
-        <v>0.3666666743874887</v>
+        <v>0.366666674387489</v>
       </c>
       <c r="AI2">
-        <v>0.3666666748072249</v>
+        <v>0.3666666748072246</v>
       </c>
       <c r="AJ2">
-        <v>0.7333333492104361</v>
+        <v>0.7333333492104359</v>
       </c>
       <c r="AK2">
-        <v>0.3666666743489842</v>
+        <v>0.3666666743489848</v>
       </c>
       <c r="AL2">
         <v>0.3666666748614589</v>
       </c>
       <c r="AM2">
-        <v>1.484120651845076E-09</v>
+        <v>1.484161479024488E-09</v>
       </c>
       <c r="AN2">
-        <v>-179.9999999988593</v>
+        <v>-179.9999999988592</v>
       </c>
       <c r="AO2">
         <v>-179.9999999981703</v>
       </c>
       <c r="AP2">
-        <v>2.878570432103091E-09</v>
+        <v>2.878607263975399E-09</v>
       </c>
       <c r="AQ2">
-        <v>-179.9999999910789</v>
+        <v>-179.9999999910787</v>
       </c>
       <c r="AR2">
         <v>179.9999999968235</v>
@@ -5649,40 +5649,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.272199217439495E-09</v>
+        <v>-2.272200962814721E-09</v>
       </c>
       <c r="O2">
-        <v>-1.904143788599209E-09</v>
+        <v>-1.904132762834685E-09</v>
       </c>
       <c r="P2">
-        <v>-3.132506384265911E-09</v>
+        <v>-3.13250703208173E-09</v>
       </c>
       <c r="Q2">
-        <v>2.272187357030036E-09</v>
+        <v>2.272189102405262E-09</v>
       </c>
       <c r="R2">
-        <v>1.904156017280334E-09</v>
+        <v>1.904146436311026E-09</v>
       </c>
       <c r="S2">
-        <v>3.132508327924384E-09</v>
+        <v>3.132510283486773E-09</v>
       </c>
       <c r="T2">
-        <v>7.0919935042141E-10</v>
+        <v>7.092035352659871E-10</v>
       </c>
       <c r="U2">
-        <v>4.349303861789564E-09</v>
+        <v>4.349316090259667E-09</v>
       </c>
       <c r="V2">
-        <v>-8.033396955548531E-10</v>
+        <v>-8.033455501270797E-10</v>
       </c>
       <c r="W2">
-        <v>-7.09194471448504E-10</v>
+        <v>-7.09198656293081E-10</v>
       </c>
       <c r="X2">
-        <v>-4.349314887314659E-09</v>
+        <v>-4.349316186856091E-09</v>
       </c>
       <c r="Y2">
-        <v>8.0335725951096E-10</v>
+        <v>8.033481537447107E-10</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -5706,10 +5706,10 @@
         <v>0.8561498316503077</v>
       </c>
       <c r="AH2">
-        <v>0.645459785903853</v>
+        <v>0.6454597859038529</v>
       </c>
       <c r="AI2">
-        <v>0.4396365303143212</v>
+        <v>0.4396365303143214</v>
       </c>
       <c r="AJ2">
         <v>0.8561498316569928</v>
@@ -5718,19 +5718,19 @@
         <v>0.6454597858855409</v>
       </c>
       <c r="AL2">
-        <v>0.4396365303501953</v>
+        <v>0.4396365303501955</v>
       </c>
       <c r="AM2">
-        <v>-3.925473815880382</v>
+        <v>-3.925473815880384</v>
       </c>
       <c r="AN2">
-        <v>-153.8407182488146</v>
+        <v>-153.8407182488145</v>
       </c>
       <c r="AO2">
         <v>128.6858355510057</v>
       </c>
       <c r="AP2">
-        <v>-3.925473814878244</v>
+        <v>-3.925473814878251</v>
       </c>
       <c r="AQ2">
         <v>-153.840718245323</v>
@@ -5924,40 +5924,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.272189380012766E-09</v>
+        <v>-2.272201240452371E-09</v>
       </c>
       <c r="O2">
-        <v>-1.904142246968138E-09</v>
+        <v>-1.904164201661341E-09</v>
       </c>
       <c r="P2">
-        <v>-3.132516785663795E-09</v>
+        <v>-3.132509635459936E-09</v>
       </c>
       <c r="Q2">
-        <v>2.272189380042912E-09</v>
+        <v>2.272189102405262E-09</v>
       </c>
       <c r="R2">
-        <v>1.904160061158417E-09</v>
+        <v>1.904165646667577E-09</v>
       </c>
       <c r="S2">
-        <v>3.132517433690635E-09</v>
+        <v>3.132507032292753E-09</v>
       </c>
       <c r="T2">
-        <v>7.091946103015332E-10</v>
+        <v>7.091994892402341E-10</v>
       </c>
       <c r="U2">
-        <v>4.349328463983553E-09</v>
+        <v>4.349317680308665E-09</v>
       </c>
       <c r="V2">
-        <v>-8.033533602616969E-10</v>
+        <v>-8.033422989330574E-10</v>
       </c>
       <c r="W2">
-        <v>-7.091946102673288E-10</v>
+        <v>-7.091986562930797E-10</v>
       </c>
       <c r="X2">
-        <v>-4.349323120324604E-09</v>
+        <v>-4.349306751140567E-09</v>
       </c>
       <c r="Y2">
-        <v>8.033592150733514E-10</v>
+        <v>8.033455503665077E-10</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -5978,34 +5978,34 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.8561498316503078</v>
+        <v>0.8561498316503074</v>
       </c>
       <c r="AH2">
-        <v>0.6454597859038528</v>
+        <v>0.6454597859038532</v>
       </c>
       <c r="AI2">
-        <v>0.4396365303143212</v>
+        <v>0.4396365303143215</v>
       </c>
       <c r="AJ2">
-        <v>0.8561498316569929</v>
+        <v>0.8561498316569924</v>
       </c>
       <c r="AK2">
-        <v>0.6454597858855405</v>
+        <v>0.6454597858855416</v>
       </c>
       <c r="AL2">
-        <v>0.4396365303501956</v>
+        <v>0.4396365303501958</v>
       </c>
       <c r="AM2">
-        <v>-3.925473815880379</v>
+        <v>-3.925473815880358</v>
       </c>
       <c r="AN2">
-        <v>-153.8407182488146</v>
+        <v>-153.8407182488145</v>
       </c>
       <c r="AO2">
         <v>128.6858355510057</v>
       </c>
       <c r="AP2">
-        <v>-3.92547381487824</v>
+        <v>-3.925473814878226</v>
       </c>
       <c r="AQ2">
         <v>-153.840718245323</v>
@@ -6199,40 +6199,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.444453331098301E-09</v>
+        <v>-2.444443857195158E-09</v>
       </c>
       <c r="O2">
-        <v>-6.111046481639845E-10</v>
+        <v>-6.111085956236261E-10</v>
       </c>
       <c r="P2">
-        <v>-6.111125436919985E-10</v>
+        <v>-6.111062277565679E-10</v>
       </c>
       <c r="Q2">
-        <v>2.44445017323126E-09</v>
+        <v>2.444448594247403E-09</v>
       </c>
       <c r="R2">
-        <v>6.111117542960412E-10</v>
+        <v>6.111101753121861E-10</v>
       </c>
       <c r="S2">
-        <v>6.111157023644172E-10</v>
+        <v>6.111046494774113E-10</v>
       </c>
       <c r="T2">
-        <v>-6.315933872496035E-15</v>
+        <v>1.557359876067895E-21</v>
       </c>
       <c r="U2">
-        <v>3.175418642475594E-09</v>
+        <v>3.175421800443308E-09</v>
       </c>
       <c r="V2">
-        <v>-3.175421803580853E-09</v>
+        <v>-3.175418645613135E-09</v>
       </c>
       <c r="W2">
-        <v>9.473961078830442E-15</v>
+        <v>3.158025648591788E-15</v>
       </c>
       <c r="X2">
         <v>-3.175424957994575E-09</v>
       </c>
       <c r="Y2">
-        <v>3.17542180399729E-09</v>
+        <v>3.175421803997287E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -6256,10 +6256,10 @@
         <v>0.6666666666635035</v>
       </c>
       <c r="AH2">
-        <v>0.3333333331670287</v>
+        <v>0.3333333331670288</v>
       </c>
       <c r="AI2">
-        <v>0.3333333334964818</v>
+        <v>0.3333333334964815</v>
       </c>
       <c r="AJ2">
         <v>0.66666666669096</v>
@@ -6268,10 +6268,10 @@
         <v>0.3333333331386026</v>
       </c>
       <c r="AL2">
-        <v>0.3333333335523633</v>
+        <v>0.3333333335523627</v>
       </c>
       <c r="AM2">
-        <v>-3.648184549803274E-11</v>
+        <v>-3.650325116654125E-11</v>
       </c>
       <c r="AN2">
         <v>-179.9999999981412</v>
@@ -6280,13 +6280,13 @@
         <v>179.9999999980558</v>
       </c>
       <c r="AP2">
-        <v>1.357946260679598E-09</v>
+        <v>1.357922999456706E-09</v>
       </c>
       <c r="AQ2">
         <v>-179.9999999844856</v>
       </c>
       <c r="AR2">
-        <v>179.9999999871891</v>
+        <v>179.999999987189</v>
       </c>
     </row>
   </sheetData>
@@ -6393,16 +6393,16 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0.4028253110876386</v>
+        <v>0.4028253110876379</v>
       </c>
       <c r="O2">
-        <v>0.4028253110894432</v>
+        <v>0.4028253110894425</v>
       </c>
       <c r="P2">
-        <v>-25.8807585799728</v>
+        <v>-25.88075857997278</v>
       </c>
       <c r="Q2">
-        <v>-25.88075857298007</v>
+        <v>-25.88075857298004</v>
       </c>
     </row>
   </sheetData>
@@ -6590,40 +6590,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-2.444453331098301E-09</v>
+        <v>-2.444443857195158E-09</v>
       </c>
       <c r="O2">
-        <v>-6.111046481639845E-10</v>
+        <v>-6.111085956236261E-10</v>
       </c>
       <c r="P2">
-        <v>-6.111125436919985E-10</v>
+        <v>-6.111062277565679E-10</v>
       </c>
       <c r="Q2">
-        <v>2.44445017323126E-09</v>
+        <v>2.444448594247403E-09</v>
       </c>
       <c r="R2">
-        <v>6.111117542960412E-10</v>
+        <v>6.111101753121861E-10</v>
       </c>
       <c r="S2">
-        <v>6.111157023644172E-10</v>
+        <v>6.111046494774113E-10</v>
       </c>
       <c r="T2">
-        <v>-6.315933872496035E-15</v>
+        <v>1.557359876067895E-21</v>
       </c>
       <c r="U2">
-        <v>3.175418642475594E-09</v>
+        <v>3.175421800443308E-09</v>
       </c>
       <c r="V2">
-        <v>-3.175421803580853E-09</v>
+        <v>-3.175418645613135E-09</v>
       </c>
       <c r="W2">
-        <v>9.473961078830442E-15</v>
+        <v>3.158025648591788E-15</v>
       </c>
       <c r="X2">
         <v>-3.175424957994575E-09</v>
       </c>
       <c r="Y2">
-        <v>3.17542180399729E-09</v>
+        <v>3.175421803997287E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -6647,10 +6647,10 @@
         <v>0.6666666666635035</v>
       </c>
       <c r="AH2">
-        <v>0.3333333331670287</v>
+        <v>0.3333333331670288</v>
       </c>
       <c r="AI2">
-        <v>0.3333333334964818</v>
+        <v>0.3333333334964815</v>
       </c>
       <c r="AJ2">
         <v>0.66666666669096</v>
@@ -6659,10 +6659,10 @@
         <v>0.3333333331386026</v>
       </c>
       <c r="AL2">
-        <v>0.3333333335523633</v>
+        <v>0.3333333335523627</v>
       </c>
       <c r="AM2">
-        <v>-3.648184549803274E-11</v>
+        <v>-3.650325116654125E-11</v>
       </c>
       <c r="AN2">
         <v>-179.9999999981412</v>
@@ -6671,13 +6671,13 @@
         <v>179.9999999980558</v>
       </c>
       <c r="AP2">
-        <v>1.357946260679598E-09</v>
+        <v>1.357922999456706E-09</v>
       </c>
       <c r="AQ2">
         <v>-179.9999999844856</v>
       </c>
       <c r="AR2">
-        <v>179.9999999871891</v>
+        <v>179.999999987189</v>
       </c>
     </row>
   </sheetData>
@@ -6865,40 +6865,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-1.9416747209887E-09</v>
+        <v>-1.941667220680918E-09</v>
       </c>
       <c r="O2">
-        <v>-1.538360062928693E-09</v>
+        <v>-1.538359891113095E-09</v>
       </c>
       <c r="P2">
-        <v>-2.506386166650113E-09</v>
+        <v>-2.506379310540052E-09</v>
       </c>
       <c r="Q2">
-        <v>1.941673026471089E-09</v>
+        <v>1.941673572909977E-09</v>
       </c>
       <c r="R2">
-        <v>1.538365991986194E-09</v>
+        <v>1.538361778900874E-09</v>
       </c>
       <c r="S2">
-        <v>2.506385258960146E-09</v>
+        <v>2.506382598178588E-09</v>
       </c>
       <c r="T2">
-        <v>5.588848233461689E-10</v>
+        <v>5.588879718083896E-10</v>
       </c>
       <c r="U2">
-        <v>3.623746713270969E-09</v>
+        <v>3.623751202745867E-09</v>
       </c>
       <c r="V2">
-        <v>-8.29287115192972E-10</v>
+        <v>-8.292894477925289E-10</v>
       </c>
       <c r="W2">
-        <v>-5.588828880694259E-10</v>
+        <v>-5.588883929619287E-10</v>
       </c>
       <c r="X2">
-        <v>-3.623748438635648E-09</v>
+        <v>-3.623748876871076E-09</v>
       </c>
       <c r="Y2">
-        <v>8.292827168319983E-10</v>
+        <v>8.292911541123508E-10</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -6925,19 +6925,19 @@
         <v>0.5655462792825743</v>
       </c>
       <c r="AI2">
-        <v>0.3792589156706163</v>
+        <v>0.3792589156706164</v>
       </c>
       <c r="AJ2">
-        <v>0.7679592756256418</v>
+        <v>0.7679592756256421</v>
       </c>
       <c r="AK2">
-        <v>0.5655462792745894</v>
+        <v>0.565546279274589</v>
       </c>
       <c r="AL2">
-        <v>0.3792589157297774</v>
+        <v>0.3792589157297773</v>
       </c>
       <c r="AM2">
-        <v>-3.793471525611841</v>
+        <v>-3.793471525611848</v>
       </c>
       <c r="AN2">
         <v>-155.6266320097133</v>
@@ -6946,13 +6946,13 @@
         <v>131.4656840130515</v>
       </c>
       <c r="AP2">
-        <v>-3.793471524370576</v>
+        <v>-3.79347152437057</v>
       </c>
       <c r="AQ2">
-        <v>-155.626632003633</v>
+        <v>-155.6266320036331</v>
       </c>
       <c r="AR2">
-        <v>131.4656840149959</v>
+        <v>131.4656840149958</v>
       </c>
     </row>
   </sheetData>
@@ -7140,40 +7140,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-1.9416747209887E-09</v>
+        <v>-1.941667220680918E-09</v>
       </c>
       <c r="O2">
-        <v>-1.538360062928693E-09</v>
+        <v>-1.538359891113095E-09</v>
       </c>
       <c r="P2">
-        <v>-2.506386166650113E-09</v>
+        <v>-2.506379310540052E-09</v>
       </c>
       <c r="Q2">
-        <v>1.941673026471089E-09</v>
+        <v>1.941673572909977E-09</v>
       </c>
       <c r="R2">
-        <v>1.538365991986194E-09</v>
+        <v>1.538361778900874E-09</v>
       </c>
       <c r="S2">
-        <v>2.506385258960146E-09</v>
+        <v>2.506382598178588E-09</v>
       </c>
       <c r="T2">
-        <v>5.588848233461689E-10</v>
+        <v>5.588879718083896E-10</v>
       </c>
       <c r="U2">
-        <v>3.623746713270969E-09</v>
+        <v>3.623751202745867E-09</v>
       </c>
       <c r="V2">
-        <v>-8.29287115192972E-10</v>
+        <v>-8.292894477925289E-10</v>
       </c>
       <c r="W2">
-        <v>-5.588828880694259E-10</v>
+        <v>-5.588883929619287E-10</v>
       </c>
       <c r="X2">
-        <v>-3.623748438635648E-09</v>
+        <v>-3.623748876871076E-09</v>
       </c>
       <c r="Y2">
-        <v>8.292827168319983E-10</v>
+        <v>8.292911541123508E-10</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -7200,19 +7200,19 @@
         <v>0.5655462792825743</v>
       </c>
       <c r="AI2">
-        <v>0.3792589156706163</v>
+        <v>0.3792589156706164</v>
       </c>
       <c r="AJ2">
-        <v>0.7679592756256418</v>
+        <v>0.7679592756256421</v>
       </c>
       <c r="AK2">
-        <v>0.5655462792745894</v>
+        <v>0.565546279274589</v>
       </c>
       <c r="AL2">
-        <v>0.3792589157297774</v>
+        <v>0.3792589157297773</v>
       </c>
       <c r="AM2">
-        <v>-3.793471525611841</v>
+        <v>-3.793471525611848</v>
       </c>
       <c r="AN2">
         <v>-155.6266320097133</v>
@@ -7221,13 +7221,13 @@
         <v>131.4656840130515</v>
       </c>
       <c r="AP2">
-        <v>-3.793471524370576</v>
+        <v>-3.79347152437057</v>
       </c>
       <c r="AQ2">
-        <v>-155.626632003633</v>
+        <v>-155.6266320036331</v>
       </c>
       <c r="AR2">
-        <v>131.4656840149959</v>
+        <v>131.4656840149958</v>
       </c>
     </row>
   </sheetData>
@@ -7334,16 +7334,16 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0.4028253110876382</v>
+        <v>0.4028253110876389</v>
       </c>
       <c r="O2">
-        <v>0.4028253110894427</v>
+        <v>0.4028253110894437</v>
       </c>
       <c r="P2">
-        <v>-25.88075857997283</v>
+        <v>-25.88075857997272</v>
       </c>
       <c r="Q2">
-        <v>-25.8807585729801</v>
+        <v>-25.88075857297997</v>
       </c>
     </row>
   </sheetData>
@@ -7682,16 +7682,16 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0.335459083046671</v>
+        <v>0.3354590830466712</v>
       </c>
       <c r="O2">
-        <v>0.3354590830702972</v>
+        <v>0.3354590830702975</v>
       </c>
       <c r="P2">
-        <v>-27.0248837607183</v>
+        <v>-27.02488376071819</v>
       </c>
       <c r="Q2">
-        <v>-27.02488374970902</v>
+        <v>-27.0248837497089</v>
       </c>
     </row>
   </sheetData>
@@ -7798,16 +7798,16 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0.335459083046671</v>
+        <v>0.3354590830466712</v>
       </c>
       <c r="O2">
-        <v>0.3354590830702972</v>
+        <v>0.3354590830702975</v>
       </c>
       <c r="P2">
-        <v>-27.0248837607183</v>
+        <v>-27.02488376071819</v>
       </c>
       <c r="Q2">
-        <v>-27.02488374970902</v>
+        <v>-27.0248837497089</v>
       </c>
     </row>
   </sheetData>
@@ -7992,40 +7992,40 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>-5.210646841688311E-15</v>
+        <v>-1.563194052506505E-14</v>
       </c>
       <c r="O2">
-        <v>1.302657326177901E-14</v>
+        <v>1.823722009817462E-14</v>
       </c>
       <c r="P2">
-        <v>1.042124915016491E-14</v>
+        <v>-5.210691387485859E-15</v>
       </c>
       <c r="Q2">
-        <v>-1.042129368337674E-14</v>
+        <v>6.021281206264993E-29</v>
       </c>
       <c r="R2">
-        <v>-2.60485133718621E-15</v>
+        <v>-1.042082159158347E-14</v>
       </c>
       <c r="S2">
-        <v>-1.563146774185772E-14</v>
+        <v>5.211119636388206E-15</v>
       </c>
       <c r="T2">
-        <v>-5.210646841688432E-15</v>
+        <v>-5.210646841688551E-15</v>
       </c>
       <c r="U2">
-        <v>5.763392256573189E-09</v>
+        <v>5.763381835279509E-09</v>
       </c>
       <c r="V2">
-        <v>-5.763397471383004E-09</v>
+        <v>-5.763392260736157E-09</v>
       </c>
       <c r="W2">
-        <v>-1.238462563867077E-28</v>
+        <v>-5.210646841688372E-15</v>
       </c>
       <c r="X2">
-        <v>-5.76338444011703E-09</v>
+        <v>-5.763384440117028E-09</v>
       </c>
       <c r="Y2">
-        <v>5.763402682515742E-09</v>
+        <v>5.763387050575207E-09</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -8046,37 +8046,37 @@
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>1.100000023808766</v>
+        <v>1.100000023808765</v>
       </c>
       <c r="AG2">
-        <v>0.550000011705747</v>
+        <v>0.5500000117057469</v>
       </c>
       <c r="AH2">
-        <v>0.5500000121030189</v>
+        <v>0.5500000121030186</v>
       </c>
       <c r="AI2">
         <v>1.100000023808766</v>
       </c>
       <c r="AJ2">
-        <v>0.5500000116593775</v>
+        <v>0.5500000116593773</v>
       </c>
       <c r="AK2">
-        <v>0.5500000121493877</v>
+        <v>0.5500000121493874</v>
       </c>
       <c r="AL2">
-        <v>6.678285403174462E-13</v>
+        <v>6.589360977838192E-13</v>
       </c>
       <c r="AM2">
-        <v>-179.9999999995569</v>
+        <v>-179.9999999995568</v>
       </c>
       <c r="AN2">
         <v>179.9999999995499</v>
       </c>
       <c r="AO2">
-        <v>6.809008569417797E-13</v>
+        <v>6.620943826402659E-13</v>
       </c>
       <c r="AP2">
-        <v>-179.9999999952996</v>
+        <v>-179.9999999952995</v>
       </c>
       <c r="AQ2">
         <v>179.9999999952925</v>

</xml_diff>